<commit_message>
Added free text guidance and redid feature types
Added guidance for free text fields, that is description and comments across all tables. And, changed feature types to be all lower-case, so it is either i, d, or c, not I.
</commit_message>
<xml_diff>
--- a/template/collection-sheet.xlsx
+++ b/template/collection-sheet.xlsx
@@ -975,54 +975,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>345440</colOff>
-      <row>2</row>
-      <rowOff>132080</rowOff>
-    </from>
-    <to>
-      <col>36</col>
-      <colOff>421640</colOff>
-      <row>54</row>
-      <rowOff>162560</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Picture 2"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9113520" y="518160"/>
-          <a:ext cx="12237720" cy="10068560"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -1307,28 +1259,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>0)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>READ ME 1st</t>
-          </r>
+          <t>0)      READ ME 1st</t>
         </is>
       </c>
     </row>
@@ -1350,56 +1281,14 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>3)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Experiment information</t>
-          </r>
+          <t>3)      Experiment information</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>4)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Experimental unit information</t>
-          </r>
+          <t>4)      Experimental unit information</t>
         </is>
       </c>
       <c r="G6" s="4" t="n"/>
@@ -1427,56 +1316,14 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>7)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Phenotype description</t>
-          </r>
+          <t>7)      Phenotype description</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>8)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Phenotype scores</t>
-          </r>
+          <t>8)      Phenotype scores</t>
         </is>
       </c>
     </row>
@@ -1490,56 +1337,14 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <r>
-            <t>10)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>      </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Climate</t>
-          </r>
+          <t>10)      Climate</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <r>
-            <t xml:space="preserve">11) </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Times New Roman"/>
-              <family val="1"/>
-              <color theme="1"/>
-              <sz val="7"/>
-            </rPr>
-            <t>  </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <family val="2"/>
-              <color theme="1"/>
-              <sz val="11"/>
-              <scheme val="minor"/>
-            </rPr>
-            <t>Management</t>
-          </r>
+          <t>11)   Management</t>
         </is>
       </c>
     </row>
@@ -1658,14 +1463,14 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>The info required in each sheet was organised according with the Database Setup diagram on the right.</t>
+          <t>The first column of each sheet is its ID. IDs can only hold the letters a-z and A-Z, the digits 0-9 and _ (no spaces, no -, and no letters with accents).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>NN means the column cannot be empty, and the key means the ID must be unique</t>
+          <t>IDs have to be unique within their sheet, and upper and lower case do not count as different: hedin_2 and Hedin_2 are the same ID.</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1701,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>With 'c' meaning any text can be placed there, 'I' only whole numbers, and 'd' any real numbers</t>
+          <t>With 'c' meaning any text can be placed there, 'i' only whole numbers, and 'd' any real numbers. Types are written in lower case.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1722,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>With Type 'd' or 'I', Vocabulary is given as a range of two numbers, within which the feature is valid, as 'min..max'. It is ends-inclusive.</t>
+          <t>With Type 'd' or 'i', Vocabulary is given as a range of two numbers, within which the feature is valid, as 'min..max'. It is ends-inclusive.</t>
         </is>
       </c>
     </row>
@@ -1931,14 +1736,14 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>(FTID1=value1;FTID2;value2;…;FTIDn=valuen)</t>
+          <t>(FTID1=value1;FTID2=value2;...;FTIDn=valuen)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>With FTID1, FTID2,…, FTIDn matching the feature IDs in FT table perfectly, and value1, value2,…, valuen confirmed to be valid values from the definition of the feature</t>
+          <t>With FTID1, FTID2, ..., FTIDn matching the feature IDs in FT table perfectly, and value1, value2, ..., valuen confirmed to be valid values from the definition of the feature</t>
         </is>
       </c>
     </row>
@@ -2059,7 +1864,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2130,7 +1934,7 @@
       </c>
       <c r="E2" s="52" t="inlineStr">
         <is>
-          <t>Description of climate covariate and how it is scored or measured</t>
+          <t>What is measured, at which height or depth, how often it is read, and how the value is calculated. Nothing about one experiment, such as the weather station or its distance (required)</t>
         </is>
       </c>
       <c r="F2" s="52" t="n"/>
@@ -2245,7 +2049,11 @@
           <t>Climate score (Numeric only, only "." (dots), no "," (commas))</t>
         </is>
       </c>
-      <c r="G2" s="26" t="n"/>
+      <c r="G2" s="62" t="inlineStr">
+        <is>
+          <t>Something about this one measurement that a reader should know</t>
+        </is>
+      </c>
       <c r="H2" s="27" t="n"/>
       <c r="I2" s="29" t="n"/>
       <c r="J2" s="29" t="n"/>
@@ -2335,7 +2143,7 @@
       </c>
       <c r="D2" s="51" t="inlineStr">
         <is>
-          <t>Longer description of treatment</t>
+          <t>The product or active ingredient, how it was applied, and why. The amount goes in Dosage</t>
         </is>
       </c>
       <c r="E2" s="50" t="inlineStr">
@@ -2348,7 +2156,11 @@
           <t>Date of treatment</t>
         </is>
       </c>
-      <c r="G2" s="21" t="n"/>
+      <c r="G2" s="53" t="inlineStr">
+        <is>
+          <t>Deviations from the plan</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2452,7 +2264,11 @@
           <t>Who maintains the variety</t>
         </is>
       </c>
-      <c r="H2" s="52" t="n"/>
+      <c r="H2" s="52" t="inlineStr">
+        <is>
+          <t>What is known about the material that no column holds, such as pedigree, breeding history or notable traits</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2535,7 +2351,11 @@
           <t>SLID of parent</t>
         </is>
       </c>
-      <c r="F2" s="52" t="n"/>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>Seed quality and handling, such as germination or seed treatment</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2655,7 +2475,7 @@
       </c>
       <c r="G2" s="78" t="inlineStr">
         <is>
-          <t>Description of trial in plain text</t>
+          <t>Site (address and field) or facility, growing conditions, trial size, plot layout, design and number of replicates, what the blocks are, any irrigation, and which factors are tested</t>
         </is>
       </c>
       <c r="H2" s="76" t="inlineStr">
@@ -2670,7 +2490,7 @@
       </c>
       <c r="J2" s="85" t="inlineStr">
         <is>
-          <t>Any comments</t>
+          <t>Events that affected the whole experiment</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2612,11 @@
           <t>Row (Integer)</t>
         </is>
       </c>
-      <c r="I2" s="52" t="n"/>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Something that happened to this unit</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2848,7 +2672,7 @@
       </c>
       <c r="B2" s="52" t="inlineStr">
         <is>
-          <t>Can be "c" for text, "I" for integer, or "d" for double, that is any non-integer real number</t>
+          <t>Kind of value, in lower case: "c" for text, "i" for whole numbers, or "d" for real numbers. Empty means "c"</t>
         </is>
       </c>
       <c r="C2" s="52" t="inlineStr">
@@ -2858,12 +2682,12 @@
       </c>
       <c r="D2" s="52" t="inlineStr">
         <is>
-          <t>Which values are allowed. For Type="c", a semicolon (;) separated list with no spaces (val1;val2) means only values val1 and val2 are allowed, and val3 would be an error. For Type="I" or Type="d", Vocabulary defines a range of two numbers, within which the feature is valid. It is given as two numbers, ends-inclusive, as min..max</t>
+          <t>Which values are allowed. For Type="c", a semicolon (;) separated list with no spaces (val1;val2) means only values val1 and val2 are allowed, and val3 would be an error. For Type="i" or Type="d", Vocabulary defines a range of two numbers, within which the feature is valid. It is given as two numbers, ends-inclusive, as min..max</t>
         </is>
       </c>
       <c r="E2" s="52" t="inlineStr">
         <is>
-          <t>A short description of what the feature is (required)</t>
+          <t>What the feature is and what its values mean, without tying it to units or to scores (required)</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2753,7 @@
       </c>
       <c r="D2" s="52" t="inlineStr">
         <is>
-          <t>Description of intervention system in trial, including all intervention categories</t>
+          <t>The intervention system, with every level defined concretely: what was done, how much and when, and which level is the control (required)</t>
         </is>
       </c>
       <c r="E2" s="21" t="n"/>
@@ -3006,7 +2830,7 @@
       </c>
       <c r="E2" s="69" t="inlineStr">
         <is>
-          <t>Description of the trait and how it is scored (Required)</t>
+          <t>What is measured, on which part of the plant, at which growth stage, with what, on how many plants and how they are chosen, how the score is calculated, and what every code means (required)</t>
         </is>
       </c>
       <c r="F2" s="69" t="n"/>
@@ -3118,7 +2942,11 @@
           <t>Name of person who scored phenotype</t>
         </is>
       </c>
-      <c r="H2" s="65" t="n"/>
+      <c r="H2" s="63" t="inlineStr">
+        <is>
+          <t>Something about this one score that a reader should know</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="14.25" customFormat="1" customHeight="1" s="3"/>
     <row r="4" ht="14.25" customFormat="1" customHeight="1" s="3"/>

</xml_diff>